<commit_message>
minor updeate to workflow
</commit_message>
<xml_diff>
--- a/docs/excel_files/Ricks Music progress.xlsx
+++ b/docs/excel_files/Ricks Music progress.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MusicProcessing\docs\excel_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18EB7741-0B0D-4FA1-8BDC-93D6557D708A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE84A0F8-F95E-4C0C-B393-AD57A92A32D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="23016" yWindow="12768" windowWidth="23256" windowHeight="12576" activeTab="4" xr2:uid="{D1BCA01E-EFE2-441C-AE68-802A69D25AC4}"/>
+    <workbookView xWindow="23016" yWindow="12768" windowWidth="23256" windowHeight="12576" activeTab="5" xr2:uid="{D1BCA01E-EFE2-441C-AE68-802A69D25AC4}"/>
   </bookViews>
   <sheets>
     <sheet name="#" sheetId="4" r:id="rId1"/>
@@ -18,12 +18,14 @@
     <sheet name="B" sheetId="5" r:id="rId3"/>
     <sheet name="C" sheetId="6" r:id="rId4"/>
     <sheet name="D" sheetId="17" r:id="rId5"/>
-    <sheet name="H" sheetId="11" r:id="rId6"/>
-    <sheet name="J" sheetId="13" r:id="rId7"/>
-    <sheet name="R" sheetId="15" r:id="rId8"/>
-    <sheet name="S" sheetId="14" r:id="rId9"/>
-    <sheet name="T" sheetId="18" r:id="rId10"/>
-    <sheet name="template" sheetId="16" r:id="rId11"/>
+    <sheet name="E" sheetId="19" r:id="rId6"/>
+    <sheet name="H" sheetId="11" r:id="rId7"/>
+    <sheet name="J" sheetId="13" r:id="rId8"/>
+    <sheet name="O" sheetId="20" r:id="rId9"/>
+    <sheet name="R" sheetId="15" r:id="rId10"/>
+    <sheet name="S" sheetId="14" r:id="rId11"/>
+    <sheet name="T" sheetId="18" r:id="rId12"/>
+    <sheet name="template" sheetId="16" r:id="rId13"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="992" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1190" uniqueCount="86">
   <si>
     <t>NA</t>
   </si>
@@ -258,6 +260,51 @@
   <si>
     <t>David Wilcox</t>
   </si>
+  <si>
+    <t>Dire Straits</t>
+  </si>
+  <si>
+    <t>Dixie Chicks</t>
+  </si>
+  <si>
+    <t>Dolly Parton</t>
+  </si>
+  <si>
+    <t>Dwight Yoakam</t>
+  </si>
+  <si>
+    <t>Double Trouble</t>
+  </si>
+  <si>
+    <t>Duffy</t>
+  </si>
+  <si>
+    <t>Ed Sheeran</t>
+  </si>
+  <si>
+    <t>Electric Light Orchestra</t>
+  </si>
+  <si>
+    <t>Elle King</t>
+  </si>
+  <si>
+    <t>Elton John</t>
+  </si>
+  <si>
+    <t>Elvis Presley</t>
+  </si>
+  <si>
+    <t>Eric Clapton</t>
+  </si>
+  <si>
+    <t>Eva Cassidy</t>
+  </si>
+  <si>
+    <t>Olivia Newton John</t>
+  </si>
+  <si>
+    <t>at a single man</t>
+  </si>
 </sst>
 </file>
 
@@ -326,7 +373,55 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="57">
+  <dxfs count="63">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i/>
+      </font>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -1262,24 +1357,24 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:XFD3">
-    <cfRule type="cellIs" dxfId="56" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="62" priority="4" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="55" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="61" priority="5" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="54" priority="6">
+    <cfRule type="expression" dxfId="60" priority="6">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O2:O3">
-    <cfRule type="cellIs" dxfId="53" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="59" priority="1" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="52" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="58" priority="2" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="51" priority="3">
+    <cfRule type="expression" dxfId="57" priority="3">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1288,6 +1383,1398 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88E4E354-CC46-4D69-85EF-A6DDA23BD060}">
+  <dimension ref="A1:P33"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="27.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.28515625" customWidth="1"/>
+    <col min="4" max="4" width="9" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.28515625" customWidth="1"/>
+    <col min="13" max="13" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="8.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" s="3" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+      <c r="H3" s="1"/>
+      <c r="I3" s="1"/>
+      <c r="J3" s="1"/>
+      <c r="K3" s="1"/>
+      <c r="L3" s="1"/>
+      <c r="M3" s="1"/>
+      <c r="N3" s="1"/>
+      <c r="O3" s="1"/>
+      <c r="P3" s="1"/>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+      <c r="J4" s="1"/>
+      <c r="K4" s="1"/>
+      <c r="L4" s="1"/>
+      <c r="M4" s="1"/>
+      <c r="N4" s="1"/>
+      <c r="O4" s="1"/>
+      <c r="P4" s="1"/>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
+      <c r="J5" s="1"/>
+      <c r="K5" s="1"/>
+      <c r="L5" s="1"/>
+      <c r="M5" s="1"/>
+      <c r="N5" s="1"/>
+      <c r="O5" s="1"/>
+      <c r="P5" s="1"/>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
+      <c r="N6" s="1"/>
+      <c r="O6" s="1"/>
+      <c r="P6" s="1"/>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A7" s="1"/>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+      <c r="J7" s="1"/>
+      <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
+      <c r="N7" s="1"/>
+      <c r="O7" s="1"/>
+      <c r="P7" s="1"/>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A8" s="1"/>
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="1"/>
+      <c r="J8" s="1"/>
+      <c r="K8" s="1"/>
+      <c r="L8" s="1"/>
+      <c r="M8" s="1"/>
+      <c r="N8" s="1"/>
+      <c r="O8" s="1"/>
+      <c r="P8" s="1"/>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A9" s="1"/>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1"/>
+      <c r="H9" s="1"/>
+      <c r="I9" s="1"/>
+      <c r="J9" s="1"/>
+      <c r="K9" s="1"/>
+      <c r="L9" s="1"/>
+      <c r="M9" s="1"/>
+      <c r="N9" s="1"/>
+      <c r="O9" s="1"/>
+      <c r="P9" s="1"/>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A10" s="1"/>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="1"/>
+      <c r="J10" s="1"/>
+      <c r="K10" s="1"/>
+      <c r="L10" s="1"/>
+      <c r="M10" s="1"/>
+      <c r="N10" s="1"/>
+      <c r="O10" s="1"/>
+      <c r="P10" s="1"/>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A11" s="1"/>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1"/>
+      <c r="H11" s="1"/>
+      <c r="I11" s="1"/>
+      <c r="J11" s="1"/>
+      <c r="K11" s="1"/>
+      <c r="L11" s="1"/>
+      <c r="M11" s="1"/>
+      <c r="N11" s="1"/>
+      <c r="O11" s="1"/>
+      <c r="P11" s="1"/>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A12" s="1"/>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="1"/>
+      <c r="H12" s="1"/>
+      <c r="I12" s="1"/>
+      <c r="J12" s="1"/>
+      <c r="K12" s="1"/>
+      <c r="L12" s="1"/>
+      <c r="M12" s="1"/>
+      <c r="N12" s="1"/>
+      <c r="O12" s="1"/>
+      <c r="P12" s="1"/>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A13" s="1"/>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="1"/>
+      <c r="H13" s="1"/>
+      <c r="I13" s="1"/>
+      <c r="J13" s="1"/>
+      <c r="K13" s="1"/>
+      <c r="L13" s="1"/>
+      <c r="M13" s="1"/>
+      <c r="N13" s="1"/>
+      <c r="O13" s="1"/>
+      <c r="P13" s="1"/>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A14" s="1"/>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1"/>
+      <c r="H14" s="1"/>
+      <c r="I14" s="1"/>
+      <c r="J14" s="1"/>
+      <c r="K14" s="1"/>
+      <c r="L14" s="1"/>
+      <c r="M14" s="1"/>
+      <c r="N14" s="1"/>
+      <c r="O14" s="1"/>
+      <c r="P14" s="1"/>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A15" s="1"/>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
+      <c r="H15" s="1"/>
+      <c r="I15" s="1"/>
+      <c r="J15" s="1"/>
+      <c r="K15" s="1"/>
+      <c r="L15" s="1"/>
+      <c r="M15" s="1"/>
+      <c r="N15" s="1"/>
+      <c r="O15" s="1"/>
+      <c r="P15" s="1"/>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A16" s="1"/>
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1"/>
+      <c r="J16" s="1"/>
+      <c r="K16" s="1"/>
+      <c r="L16" s="1"/>
+      <c r="M16" s="1"/>
+      <c r="N16" s="1"/>
+      <c r="O16" s="1"/>
+      <c r="P16" s="1"/>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A17" s="1"/>
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
+      <c r="H17" s="1"/>
+      <c r="I17" s="1"/>
+      <c r="J17" s="1"/>
+      <c r="K17" s="1"/>
+      <c r="L17" s="1"/>
+      <c r="M17" s="1"/>
+      <c r="N17" s="1"/>
+      <c r="O17" s="1"/>
+      <c r="P17" s="1"/>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A18" s="1"/>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
+      <c r="G18" s="1"/>
+      <c r="H18" s="1"/>
+      <c r="I18" s="1"/>
+      <c r="J18" s="1"/>
+      <c r="K18" s="1"/>
+      <c r="L18" s="1"/>
+      <c r="M18" s="1"/>
+      <c r="N18" s="1"/>
+      <c r="O18" s="1"/>
+      <c r="P18" s="1"/>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A19" s="1"/>
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+      <c r="F19" s="1"/>
+      <c r="G19" s="1"/>
+      <c r="H19" s="1"/>
+      <c r="I19" s="1"/>
+      <c r="J19" s="1"/>
+      <c r="K19" s="1"/>
+      <c r="L19" s="1"/>
+      <c r="M19" s="1"/>
+      <c r="N19" s="1"/>
+      <c r="O19" s="1"/>
+      <c r="P19" s="1"/>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A20" s="1"/>
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
+      <c r="G20" s="1"/>
+      <c r="H20" s="1"/>
+      <c r="I20" s="1"/>
+      <c r="J20" s="1"/>
+      <c r="K20" s="1"/>
+      <c r="L20" s="1"/>
+      <c r="M20" s="1"/>
+      <c r="N20" s="1"/>
+      <c r="O20" s="1"/>
+      <c r="P20" s="1"/>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A21" s="1"/>
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1"/>
+      <c r="G21" s="1"/>
+      <c r="H21" s="1"/>
+      <c r="I21" s="1"/>
+      <c r="J21" s="1"/>
+      <c r="K21" s="1"/>
+      <c r="L21" s="1"/>
+      <c r="M21" s="1"/>
+      <c r="N21" s="1"/>
+      <c r="O21" s="1"/>
+      <c r="P21" s="1"/>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A22" s="1"/>
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+      <c r="F22" s="1"/>
+      <c r="G22" s="1"/>
+      <c r="H22" s="1"/>
+      <c r="I22" s="1"/>
+      <c r="J22" s="1"/>
+      <c r="K22" s="1"/>
+      <c r="L22" s="1"/>
+      <c r="M22" s="1"/>
+      <c r="N22" s="1"/>
+      <c r="O22" s="1"/>
+      <c r="P22" s="1"/>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A23" s="1"/>
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+      <c r="F23" s="1"/>
+      <c r="G23" s="1"/>
+      <c r="H23" s="1"/>
+      <c r="I23" s="1"/>
+      <c r="J23" s="1"/>
+      <c r="K23" s="1"/>
+      <c r="L23" s="1"/>
+      <c r="M23" s="1"/>
+      <c r="N23" s="1"/>
+      <c r="O23" s="1"/>
+      <c r="P23" s="1"/>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A24" s="1"/>
+      <c r="B24" s="1"/>
+      <c r="C24" s="1"/>
+      <c r="D24" s="1"/>
+      <c r="E24" s="1"/>
+      <c r="F24" s="1"/>
+      <c r="G24" s="1"/>
+      <c r="H24" s="1"/>
+      <c r="I24" s="1"/>
+      <c r="J24" s="1"/>
+      <c r="K24" s="1"/>
+      <c r="L24" s="1"/>
+      <c r="M24" s="1"/>
+      <c r="N24" s="1"/>
+      <c r="O24" s="1"/>
+      <c r="P24" s="1"/>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A25" s="1"/>
+      <c r="B25" s="1"/>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
+      <c r="F25" s="1"/>
+      <c r="G25" s="1"/>
+      <c r="H25" s="1"/>
+      <c r="I25" s="1"/>
+      <c r="J25" s="1"/>
+      <c r="K25" s="1"/>
+      <c r="L25" s="1"/>
+      <c r="M25" s="1"/>
+      <c r="N25" s="1"/>
+      <c r="O25" s="1"/>
+      <c r="P25" s="1"/>
+    </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A26" s="1"/>
+      <c r="B26" s="1"/>
+      <c r="C26" s="1"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="1"/>
+      <c r="F26" s="1"/>
+      <c r="G26" s="1"/>
+      <c r="H26" s="1"/>
+      <c r="I26" s="1"/>
+      <c r="J26" s="1"/>
+      <c r="K26" s="1"/>
+      <c r="L26" s="1"/>
+      <c r="M26" s="1"/>
+      <c r="N26" s="1"/>
+      <c r="O26" s="1"/>
+      <c r="P26" s="1"/>
+    </row>
+    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A27" s="1"/>
+      <c r="B27" s="1"/>
+      <c r="C27" s="1"/>
+      <c r="D27" s="1"/>
+      <c r="E27" s="1"/>
+      <c r="F27" s="1"/>
+      <c r="G27" s="1"/>
+      <c r="H27" s="1"/>
+      <c r="I27" s="1"/>
+      <c r="J27" s="1"/>
+      <c r="K27" s="1"/>
+      <c r="L27" s="1"/>
+      <c r="M27" s="1"/>
+      <c r="N27" s="1"/>
+      <c r="O27" s="1"/>
+      <c r="P27" s="1"/>
+    </row>
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A28" s="1"/>
+      <c r="B28" s="1"/>
+      <c r="C28" s="1"/>
+      <c r="D28" s="1"/>
+      <c r="E28" s="1"/>
+      <c r="F28" s="1"/>
+      <c r="G28" s="1"/>
+      <c r="H28" s="1"/>
+      <c r="I28" s="1"/>
+      <c r="J28" s="1"/>
+      <c r="K28" s="1"/>
+      <c r="L28" s="1"/>
+      <c r="M28" s="1"/>
+      <c r="N28" s="1"/>
+      <c r="O28" s="1"/>
+      <c r="P28" s="1"/>
+    </row>
+    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A29" s="1"/>
+      <c r="B29" s="1"/>
+      <c r="C29" s="1"/>
+      <c r="D29" s="1"/>
+      <c r="E29" s="1"/>
+      <c r="F29" s="1"/>
+      <c r="G29" s="1"/>
+      <c r="H29" s="1"/>
+      <c r="I29" s="1"/>
+      <c r="J29" s="1"/>
+      <c r="K29" s="1"/>
+      <c r="L29" s="1"/>
+      <c r="M29" s="1"/>
+      <c r="N29" s="1"/>
+      <c r="O29" s="1"/>
+      <c r="P29" s="1"/>
+    </row>
+    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A30" s="1"/>
+      <c r="B30" s="1"/>
+      <c r="C30" s="1"/>
+      <c r="D30" s="1"/>
+      <c r="E30" s="1"/>
+      <c r="F30" s="1"/>
+      <c r="G30" s="1"/>
+      <c r="H30" s="1"/>
+      <c r="I30" s="1"/>
+      <c r="J30" s="1"/>
+      <c r="K30" s="1"/>
+      <c r="L30" s="1"/>
+      <c r="M30" s="1"/>
+      <c r="N30" s="1"/>
+      <c r="O30" s="1"/>
+      <c r="P30" s="1"/>
+    </row>
+    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A31" s="1"/>
+      <c r="B31" s="1"/>
+      <c r="C31" s="1"/>
+      <c r="D31" s="1"/>
+      <c r="E31" s="1"/>
+      <c r="F31" s="1"/>
+      <c r="G31" s="1"/>
+      <c r="H31" s="1"/>
+      <c r="I31" s="1"/>
+      <c r="J31" s="1"/>
+      <c r="K31" s="1"/>
+      <c r="L31" s="1"/>
+      <c r="M31" s="1"/>
+      <c r="N31" s="1"/>
+      <c r="O31" s="1"/>
+      <c r="P31" s="1"/>
+    </row>
+    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A32" s="1"/>
+      <c r="B32" s="1"/>
+      <c r="C32" s="1"/>
+      <c r="D32" s="1"/>
+      <c r="E32" s="1"/>
+      <c r="F32" s="1"/>
+      <c r="G32" s="1"/>
+      <c r="H32" s="1"/>
+      <c r="I32" s="1"/>
+      <c r="J32" s="1"/>
+      <c r="K32" s="1"/>
+      <c r="L32" s="1"/>
+      <c r="M32" s="1"/>
+      <c r="N32" s="1"/>
+      <c r="O32" s="1"/>
+      <c r="P32" s="1"/>
+    </row>
+    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A33" s="1"/>
+      <c r="B33" s="1"/>
+      <c r="C33" s="1"/>
+      <c r="D33" s="1"/>
+      <c r="E33" s="1"/>
+      <c r="F33" s="1"/>
+      <c r="G33" s="1"/>
+      <c r="H33" s="1"/>
+      <c r="I33" s="1"/>
+      <c r="J33" s="1"/>
+      <c r="K33" s="1"/>
+      <c r="L33" s="1"/>
+      <c r="M33" s="1"/>
+      <c r="N33" s="1"/>
+      <c r="O33" s="1"/>
+      <c r="P33" s="1"/>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="A2:XFD33">
+    <cfRule type="cellIs" dxfId="26" priority="1" operator="equal">
+      <formula>"No"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="25" priority="2" operator="equal">
+      <formula>"Yes"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="24" priority="3">
+      <formula>MOD(ROW(), 2) = 0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2C91933-1FED-40CE-A7F7-694A14E79AF4}">
+  <dimension ref="A1:P33"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="27.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.28515625" customWidth="1"/>
+    <col min="4" max="4" width="9" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.28515625" customWidth="1"/>
+    <col min="13" max="13" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="8.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" s="3" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+      <c r="H3" s="1"/>
+      <c r="I3" s="1"/>
+      <c r="J3" s="1"/>
+      <c r="K3" s="1"/>
+      <c r="L3" s="1"/>
+      <c r="M3" s="1"/>
+      <c r="N3" s="1"/>
+      <c r="O3" s="1"/>
+      <c r="P3" s="1"/>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+      <c r="J4" s="1"/>
+      <c r="K4" s="1"/>
+      <c r="L4" s="1"/>
+      <c r="M4" s="1"/>
+      <c r="N4" s="1"/>
+      <c r="O4" s="1"/>
+      <c r="P4" s="1"/>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
+      <c r="J5" s="1"/>
+      <c r="K5" s="1"/>
+      <c r="L5" s="1"/>
+      <c r="M5" s="1"/>
+      <c r="N5" s="1"/>
+      <c r="O5" s="1"/>
+      <c r="P5" s="1"/>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
+      <c r="N6" s="1"/>
+      <c r="O6" s="1"/>
+      <c r="P6" s="1"/>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A7" s="1"/>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+      <c r="J7" s="1"/>
+      <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
+      <c r="N7" s="1"/>
+      <c r="O7" s="1"/>
+      <c r="P7" s="1"/>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A8" s="1"/>
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="1"/>
+      <c r="J8" s="1"/>
+      <c r="K8" s="1"/>
+      <c r="L8" s="1"/>
+      <c r="M8" s="1"/>
+      <c r="N8" s="1"/>
+      <c r="O8" s="1"/>
+      <c r="P8" s="1"/>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A9" s="1"/>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1"/>
+      <c r="H9" s="1"/>
+      <c r="I9" s="1"/>
+      <c r="J9" s="1"/>
+      <c r="K9" s="1"/>
+      <c r="L9" s="1"/>
+      <c r="M9" s="1"/>
+      <c r="N9" s="1"/>
+      <c r="O9" s="1"/>
+      <c r="P9" s="1"/>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A10" s="1"/>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="1"/>
+      <c r="J10" s="1"/>
+      <c r="K10" s="1"/>
+      <c r="L10" s="1"/>
+      <c r="M10" s="1"/>
+      <c r="N10" s="1"/>
+      <c r="O10" s="1"/>
+      <c r="P10" s="1"/>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A11" s="1"/>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1"/>
+      <c r="H11" s="1"/>
+      <c r="I11" s="1"/>
+      <c r="J11" s="1"/>
+      <c r="K11" s="1"/>
+      <c r="L11" s="1"/>
+      <c r="M11" s="1"/>
+      <c r="N11" s="1"/>
+      <c r="O11" s="1"/>
+      <c r="P11" s="1"/>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A12" s="1"/>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="1"/>
+      <c r="H12" s="1"/>
+      <c r="I12" s="1"/>
+      <c r="J12" s="1"/>
+      <c r="K12" s="1"/>
+      <c r="L12" s="1"/>
+      <c r="M12" s="1"/>
+      <c r="N12" s="1"/>
+      <c r="O12" s="1"/>
+      <c r="P12" s="1"/>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A13" s="1"/>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="1"/>
+      <c r="H13" s="1"/>
+      <c r="I13" s="1"/>
+      <c r="J13" s="1"/>
+      <c r="K13" s="1"/>
+      <c r="L13" s="1"/>
+      <c r="M13" s="1"/>
+      <c r="N13" s="1"/>
+      <c r="O13" s="1"/>
+      <c r="P13" s="1"/>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A14" s="1"/>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1"/>
+      <c r="H14" s="1"/>
+      <c r="I14" s="1"/>
+      <c r="J14" s="1"/>
+      <c r="K14" s="1"/>
+      <c r="L14" s="1"/>
+      <c r="M14" s="1"/>
+      <c r="N14" s="1"/>
+      <c r="O14" s="1"/>
+      <c r="P14" s="1"/>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A15" s="1"/>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
+      <c r="H15" s="1"/>
+      <c r="I15" s="1"/>
+      <c r="J15" s="1"/>
+      <c r="K15" s="1"/>
+      <c r="L15" s="1"/>
+      <c r="M15" s="1"/>
+      <c r="N15" s="1"/>
+      <c r="O15" s="1"/>
+      <c r="P15" s="1"/>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A16" s="1"/>
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1"/>
+      <c r="J16" s="1"/>
+      <c r="K16" s="1"/>
+      <c r="L16" s="1"/>
+      <c r="M16" s="1"/>
+      <c r="N16" s="1"/>
+      <c r="O16" s="1"/>
+      <c r="P16" s="1"/>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A17" s="1"/>
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
+      <c r="H17" s="1"/>
+      <c r="I17" s="1"/>
+      <c r="J17" s="1"/>
+      <c r="K17" s="1"/>
+      <c r="L17" s="1"/>
+      <c r="M17" s="1"/>
+      <c r="N17" s="1"/>
+      <c r="O17" s="1"/>
+      <c r="P17" s="1"/>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A18" s="1"/>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
+      <c r="G18" s="1"/>
+      <c r="H18" s="1"/>
+      <c r="I18" s="1"/>
+      <c r="J18" s="1"/>
+      <c r="K18" s="1"/>
+      <c r="L18" s="1"/>
+      <c r="M18" s="1"/>
+      <c r="N18" s="1"/>
+      <c r="O18" s="1"/>
+      <c r="P18" s="1"/>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A19" s="1"/>
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+      <c r="F19" s="1"/>
+      <c r="G19" s="1"/>
+      <c r="H19" s="1"/>
+      <c r="I19" s="1"/>
+      <c r="J19" s="1"/>
+      <c r="K19" s="1"/>
+      <c r="L19" s="1"/>
+      <c r="M19" s="1"/>
+      <c r="N19" s="1"/>
+      <c r="O19" s="1"/>
+      <c r="P19" s="1"/>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A20" s="1"/>
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
+      <c r="G20" s="1"/>
+      <c r="H20" s="1"/>
+      <c r="I20" s="1"/>
+      <c r="J20" s="1"/>
+      <c r="K20" s="1"/>
+      <c r="L20" s="1"/>
+      <c r="M20" s="1"/>
+      <c r="N20" s="1"/>
+      <c r="O20" s="1"/>
+      <c r="P20" s="1"/>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A21" s="1"/>
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1"/>
+      <c r="G21" s="1"/>
+      <c r="H21" s="1"/>
+      <c r="I21" s="1"/>
+      <c r="J21" s="1"/>
+      <c r="K21" s="1"/>
+      <c r="L21" s="1"/>
+      <c r="M21" s="1"/>
+      <c r="N21" s="1"/>
+      <c r="O21" s="1"/>
+      <c r="P21" s="1"/>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A22" s="1"/>
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+      <c r="F22" s="1"/>
+      <c r="G22" s="1"/>
+      <c r="H22" s="1"/>
+      <c r="I22" s="1"/>
+      <c r="J22" s="1"/>
+      <c r="K22" s="1"/>
+      <c r="L22" s="1"/>
+      <c r="M22" s="1"/>
+      <c r="N22" s="1"/>
+      <c r="O22" s="1"/>
+      <c r="P22" s="1"/>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A23" s="1"/>
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+      <c r="F23" s="1"/>
+      <c r="G23" s="1"/>
+      <c r="H23" s="1"/>
+      <c r="I23" s="1"/>
+      <c r="J23" s="1"/>
+      <c r="K23" s="1"/>
+      <c r="L23" s="1"/>
+      <c r="M23" s="1"/>
+      <c r="N23" s="1"/>
+      <c r="O23" s="1"/>
+      <c r="P23" s="1"/>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A24" s="1"/>
+      <c r="B24" s="1"/>
+      <c r="C24" s="1"/>
+      <c r="D24" s="1"/>
+      <c r="E24" s="1"/>
+      <c r="F24" s="1"/>
+      <c r="G24" s="1"/>
+      <c r="H24" s="1"/>
+      <c r="I24" s="1"/>
+      <c r="J24" s="1"/>
+      <c r="K24" s="1"/>
+      <c r="L24" s="1"/>
+      <c r="M24" s="1"/>
+      <c r="N24" s="1"/>
+      <c r="O24" s="1"/>
+      <c r="P24" s="1"/>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A25" s="1"/>
+      <c r="B25" s="1"/>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
+      <c r="F25" s="1"/>
+      <c r="G25" s="1"/>
+      <c r="H25" s="1"/>
+      <c r="I25" s="1"/>
+      <c r="J25" s="1"/>
+      <c r="K25" s="1"/>
+      <c r="L25" s="1"/>
+      <c r="M25" s="1"/>
+      <c r="N25" s="1"/>
+      <c r="O25" s="1"/>
+      <c r="P25" s="1"/>
+    </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A26" s="1"/>
+      <c r="B26" s="1"/>
+      <c r="C26" s="1"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="1"/>
+      <c r="F26" s="1"/>
+      <c r="G26" s="1"/>
+      <c r="H26" s="1"/>
+      <c r="I26" s="1"/>
+      <c r="J26" s="1"/>
+      <c r="K26" s="1"/>
+      <c r="L26" s="1"/>
+      <c r="M26" s="1"/>
+      <c r="N26" s="1"/>
+      <c r="O26" s="1"/>
+      <c r="P26" s="1"/>
+    </row>
+    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A27" s="1"/>
+      <c r="B27" s="1"/>
+      <c r="C27" s="1"/>
+      <c r="D27" s="1"/>
+      <c r="E27" s="1"/>
+      <c r="F27" s="1"/>
+      <c r="G27" s="1"/>
+      <c r="H27" s="1"/>
+      <c r="I27" s="1"/>
+      <c r="J27" s="1"/>
+      <c r="K27" s="1"/>
+      <c r="L27" s="1"/>
+      <c r="M27" s="1"/>
+      <c r="N27" s="1"/>
+      <c r="O27" s="1"/>
+      <c r="P27" s="1"/>
+    </row>
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A28" s="1"/>
+      <c r="B28" s="1"/>
+      <c r="C28" s="1"/>
+      <c r="D28" s="1"/>
+      <c r="E28" s="1"/>
+      <c r="F28" s="1"/>
+      <c r="G28" s="1"/>
+      <c r="H28" s="1"/>
+      <c r="I28" s="1"/>
+      <c r="J28" s="1"/>
+      <c r="K28" s="1"/>
+      <c r="L28" s="1"/>
+      <c r="M28" s="1"/>
+      <c r="N28" s="1"/>
+      <c r="O28" s="1"/>
+      <c r="P28" s="1"/>
+    </row>
+    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A29" s="1"/>
+      <c r="B29" s="1"/>
+      <c r="C29" s="1"/>
+      <c r="D29" s="1"/>
+      <c r="E29" s="1"/>
+      <c r="F29" s="1"/>
+      <c r="G29" s="1"/>
+      <c r="H29" s="1"/>
+      <c r="I29" s="1"/>
+      <c r="J29" s="1"/>
+      <c r="K29" s="1"/>
+      <c r="L29" s="1"/>
+      <c r="M29" s="1"/>
+      <c r="N29" s="1"/>
+      <c r="O29" s="1"/>
+      <c r="P29" s="1"/>
+    </row>
+    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A30" s="1"/>
+      <c r="B30" s="1"/>
+      <c r="C30" s="1"/>
+      <c r="D30" s="1"/>
+      <c r="E30" s="1"/>
+      <c r="F30" s="1"/>
+      <c r="G30" s="1"/>
+      <c r="H30" s="1"/>
+      <c r="I30" s="1"/>
+      <c r="J30" s="1"/>
+      <c r="K30" s="1"/>
+      <c r="L30" s="1"/>
+      <c r="M30" s="1"/>
+      <c r="N30" s="1"/>
+      <c r="O30" s="1"/>
+      <c r="P30" s="1"/>
+    </row>
+    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A31" s="1"/>
+      <c r="B31" s="1"/>
+      <c r="C31" s="1"/>
+      <c r="D31" s="1"/>
+      <c r="E31" s="1"/>
+      <c r="F31" s="1"/>
+      <c r="G31" s="1"/>
+      <c r="H31" s="1"/>
+      <c r="I31" s="1"/>
+      <c r="J31" s="1"/>
+      <c r="K31" s="1"/>
+      <c r="L31" s="1"/>
+      <c r="M31" s="1"/>
+      <c r="N31" s="1"/>
+      <c r="O31" s="1"/>
+      <c r="P31" s="1"/>
+    </row>
+    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A32" s="1"/>
+      <c r="B32" s="1"/>
+      <c r="C32" s="1"/>
+      <c r="D32" s="1"/>
+      <c r="E32" s="1"/>
+      <c r="F32" s="1"/>
+      <c r="G32" s="1"/>
+      <c r="H32" s="1"/>
+      <c r="I32" s="1"/>
+      <c r="J32" s="1"/>
+      <c r="K32" s="1"/>
+      <c r="L32" s="1"/>
+      <c r="M32" s="1"/>
+      <c r="N32" s="1"/>
+      <c r="O32" s="1"/>
+      <c r="P32" s="1"/>
+    </row>
+    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A33" s="1"/>
+      <c r="B33" s="1"/>
+      <c r="C33" s="1"/>
+      <c r="D33" s="1"/>
+      <c r="E33" s="1"/>
+      <c r="F33" s="1"/>
+      <c r="G33" s="1"/>
+      <c r="H33" s="1"/>
+      <c r="I33" s="1"/>
+      <c r="J33" s="1"/>
+      <c r="K33" s="1"/>
+      <c r="L33" s="1"/>
+      <c r="M33" s="1"/>
+      <c r="N33" s="1"/>
+      <c r="O33" s="1"/>
+      <c r="P33" s="1"/>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="A2:XFD33">
+    <cfRule type="cellIs" dxfId="23" priority="1" operator="equal">
+      <formula>"No"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="22" priority="2" operator="equal">
+      <formula>"Yes"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="21" priority="3">
+      <formula>MOD(ROW(), 2) = 0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{773E741D-F1A5-41A0-B656-3E8F5BB0844F}">
   <dimension ref="A1:P34"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2017,7 +3504,29 @@
       <c r="P34" s="1"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A4:XFD34 A3:L3 P3:XFD3">
+  <conditionalFormatting sqref="A3:O3">
+    <cfRule type="cellIs" dxfId="20" priority="1" operator="equal">
+      <formula>"No"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="19" priority="2" operator="equal">
+      <formula>"Yes"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="18" priority="3">
+      <formula>MOD(ROW(), 2) = 0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2:P2">
+    <cfRule type="cellIs" dxfId="17" priority="4" operator="equal">
+      <formula>"No"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="16" priority="5" operator="equal">
+      <formula>"Yes"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="15" priority="6">
+      <formula>MOD(ROW(), 2) = 0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A4:XFD34">
     <cfRule type="cellIs" dxfId="14" priority="10" operator="equal">
       <formula>"No"</formula>
     </cfRule>
@@ -2028,38 +3537,14 @@
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:P2">
-    <cfRule type="cellIs" dxfId="11" priority="4" operator="equal">
+  <conditionalFormatting sqref="P2:XFD3">
+    <cfRule type="cellIs" dxfId="11" priority="7" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="8" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="6">
-      <formula>MOD(ROW(), 2) = 0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="P2:XFD2">
-    <cfRule type="cellIs" dxfId="8" priority="7" operator="equal">
-      <formula>"No"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="8" operator="equal">
-      <formula>"Yes"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="P2:XFD2">
-    <cfRule type="expression" dxfId="6" priority="9">
-      <formula>MOD(ROW(), 2) = 0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M3:O3">
-    <cfRule type="cellIs" dxfId="5" priority="1" operator="equal">
-      <formula>"No"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
-      <formula>"Yes"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="3" priority="3">
+    <cfRule type="expression" dxfId="9" priority="9">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2067,7 +3552,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4CE04A26-E0D7-4F6E-9369-31B8371FBE59}">
   <dimension ref="A1:P33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2748,13 +4233,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:XFD33">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="1" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="2" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="3">
+    <cfRule type="expression" dxfId="6" priority="3">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3333,33 +4818,33 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:XFD11">
-    <cfRule type="cellIs" dxfId="50" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="56" priority="7" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="49" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="55" priority="8" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="48" priority="9">
+    <cfRule type="expression" dxfId="54" priority="9">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O2:O11">
-    <cfRule type="cellIs" dxfId="47" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="53" priority="1" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="46" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="52" priority="2" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="45" priority="3">
+    <cfRule type="expression" dxfId="51" priority="3">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="44" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="50" priority="4" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="43" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="49" priority="5" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="42" priority="6">
+    <cfRule type="expression" dxfId="48" priority="6">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4799,24 +6284,24 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:O48 Q2:XFD48 N18:P48">
-    <cfRule type="cellIs" dxfId="41" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="47" priority="4" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="40" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="46" priority="5" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="39" priority="6">
+    <cfRule type="expression" dxfId="45" priority="6">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P2:P17">
-    <cfRule type="cellIs" dxfId="38" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="44" priority="1" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="37" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="43" priority="2" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="36" priority="3">
+    <cfRule type="expression" dxfId="42" priority="3">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5826,6 +7311,998 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:P12">
+    <cfRule type="cellIs" dxfId="41" priority="1" operator="equal">
+      <formula>"No"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="40" priority="2" operator="equal">
+      <formula>"Yes"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="39" priority="3">
+      <formula>MOD(ROW(), 2) = 0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P3:XFD12 Q2:XFD2 A13:XFD33">
+    <cfRule type="cellIs" dxfId="38" priority="10" operator="equal">
+      <formula>"No"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="37" priority="11" operator="equal">
+      <formula>"Yes"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q2:XFD2 P3:XFD12 A13:XFD33">
+    <cfRule type="expression" dxfId="36" priority="12">
+      <formula>MOD(ROW(), 2) = 0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A665A9A6-A955-425D-A292-ED453B420318}">
+  <dimension ref="A1:P31"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="27.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.28515625" customWidth="1"/>
+    <col min="4" max="4" width="9" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.28515625" customWidth="1"/>
+    <col min="13" max="13" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" s="3" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="N3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="O3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="P3" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="P4" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="M5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="N5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="O5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="P5" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="M6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="N6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="O6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="P6" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="M7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="N7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="O7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="P7" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="L8" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="M8" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="N8" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="O8" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="P8" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="M9" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="N9" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="O9" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="P9" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="K10" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="L10" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="M10" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="N10" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="O10" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="P10" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="K11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="L11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="M11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="N11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="O11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="P11" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J12" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="K12" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="L12" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="M12" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="N12" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="O12" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="P12" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A13" s="1"/>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="1"/>
+      <c r="H13" s="1"/>
+      <c r="I13" s="1"/>
+      <c r="J13" s="1"/>
+      <c r="K13" s="1"/>
+      <c r="L13" s="1"/>
+      <c r="M13" s="1"/>
+      <c r="N13" s="1"/>
+      <c r="O13" s="1"/>
+      <c r="P13" s="1"/>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A14" s="1"/>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1"/>
+      <c r="H14" s="1"/>
+      <c r="I14" s="1"/>
+      <c r="J14" s="1"/>
+      <c r="K14" s="1"/>
+      <c r="L14" s="1"/>
+      <c r="M14" s="1"/>
+      <c r="N14" s="1"/>
+      <c r="O14" s="1"/>
+      <c r="P14" s="1"/>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A15" s="1"/>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
+      <c r="H15" s="1"/>
+      <c r="I15" s="1"/>
+      <c r="J15" s="1"/>
+      <c r="K15" s="1"/>
+      <c r="L15" s="1"/>
+      <c r="M15" s="1"/>
+      <c r="N15" s="1"/>
+      <c r="O15" s="1"/>
+      <c r="P15" s="1"/>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A16" s="1"/>
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1"/>
+      <c r="J16" s="1"/>
+      <c r="K16" s="1"/>
+      <c r="L16" s="1"/>
+      <c r="M16" s="1"/>
+      <c r="N16" s="1"/>
+      <c r="O16" s="1"/>
+      <c r="P16" s="1"/>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A17" s="1"/>
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
+      <c r="H17" s="1"/>
+      <c r="I17" s="1"/>
+      <c r="J17" s="1"/>
+      <c r="K17" s="1"/>
+      <c r="L17" s="1"/>
+      <c r="M17" s="1"/>
+      <c r="N17" s="1"/>
+      <c r="O17" s="1"/>
+      <c r="P17" s="1"/>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A18" s="1"/>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
+      <c r="G18" s="1"/>
+      <c r="H18" s="1"/>
+      <c r="I18" s="1"/>
+      <c r="J18" s="1"/>
+      <c r="K18" s="1"/>
+      <c r="L18" s="1"/>
+      <c r="M18" s="1"/>
+      <c r="N18" s="1"/>
+      <c r="O18" s="1"/>
+      <c r="P18" s="1"/>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A19" s="1"/>
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+      <c r="F19" s="1"/>
+      <c r="G19" s="1"/>
+      <c r="H19" s="1"/>
+      <c r="I19" s="1"/>
+      <c r="J19" s="1"/>
+      <c r="K19" s="1"/>
+      <c r="L19" s="1"/>
+      <c r="M19" s="1"/>
+      <c r="N19" s="1"/>
+      <c r="O19" s="1"/>
+      <c r="P19" s="1"/>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A20" s="1"/>
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
+      <c r="G20" s="1"/>
+      <c r="H20" s="1"/>
+      <c r="I20" s="1"/>
+      <c r="J20" s="1"/>
+      <c r="K20" s="1"/>
+      <c r="L20" s="1"/>
+      <c r="M20" s="1"/>
+      <c r="N20" s="1"/>
+      <c r="O20" s="1"/>
+      <c r="P20" s="1"/>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A21" s="1"/>
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1"/>
+      <c r="G21" s="1"/>
+      <c r="H21" s="1"/>
+      <c r="I21" s="1"/>
+      <c r="J21" s="1"/>
+      <c r="K21" s="1"/>
+      <c r="L21" s="1"/>
+      <c r="M21" s="1"/>
+      <c r="N21" s="1"/>
+      <c r="O21" s="1"/>
+      <c r="P21" s="1"/>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A22" s="1"/>
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+      <c r="F22" s="1"/>
+      <c r="G22" s="1"/>
+      <c r="H22" s="1"/>
+      <c r="I22" s="1"/>
+      <c r="J22" s="1"/>
+      <c r="K22" s="1"/>
+      <c r="L22" s="1"/>
+      <c r="M22" s="1"/>
+      <c r="N22" s="1"/>
+      <c r="O22" s="1"/>
+      <c r="P22" s="1"/>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A23" s="1"/>
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+      <c r="F23" s="1"/>
+      <c r="G23" s="1"/>
+      <c r="H23" s="1"/>
+      <c r="I23" s="1"/>
+      <c r="J23" s="1"/>
+      <c r="K23" s="1"/>
+      <c r="L23" s="1"/>
+      <c r="M23" s="1"/>
+      <c r="N23" s="1"/>
+      <c r="O23" s="1"/>
+      <c r="P23" s="1"/>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A24" s="1"/>
+      <c r="B24" s="1"/>
+      <c r="C24" s="1"/>
+      <c r="D24" s="1"/>
+      <c r="E24" s="1"/>
+      <c r="F24" s="1"/>
+      <c r="G24" s="1"/>
+      <c r="H24" s="1"/>
+      <c r="I24" s="1"/>
+      <c r="J24" s="1"/>
+      <c r="K24" s="1"/>
+      <c r="L24" s="1"/>
+      <c r="M24" s="1"/>
+      <c r="N24" s="1"/>
+      <c r="O24" s="1"/>
+      <c r="P24" s="1"/>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A25" s="1"/>
+      <c r="B25" s="1"/>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
+      <c r="F25" s="1"/>
+      <c r="G25" s="1"/>
+      <c r="H25" s="1"/>
+      <c r="I25" s="1"/>
+      <c r="J25" s="1"/>
+      <c r="K25" s="1"/>
+      <c r="L25" s="1"/>
+      <c r="M25" s="1"/>
+      <c r="N25" s="1"/>
+      <c r="O25" s="1"/>
+      <c r="P25" s="1"/>
+    </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A26" s="1"/>
+      <c r="B26" s="1"/>
+      <c r="C26" s="1"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="1"/>
+      <c r="F26" s="1"/>
+      <c r="G26" s="1"/>
+      <c r="H26" s="1"/>
+      <c r="I26" s="1"/>
+      <c r="J26" s="1"/>
+      <c r="K26" s="1"/>
+      <c r="L26" s="1"/>
+      <c r="M26" s="1"/>
+      <c r="N26" s="1"/>
+      <c r="O26" s="1"/>
+      <c r="P26" s="1"/>
+    </row>
+    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A27" s="1"/>
+      <c r="B27" s="1"/>
+      <c r="C27" s="1"/>
+      <c r="D27" s="1"/>
+      <c r="E27" s="1"/>
+      <c r="F27" s="1"/>
+      <c r="G27" s="1"/>
+      <c r="H27" s="1"/>
+      <c r="I27" s="1"/>
+      <c r="J27" s="1"/>
+      <c r="K27" s="1"/>
+      <c r="L27" s="1"/>
+      <c r="M27" s="1"/>
+      <c r="N27" s="1"/>
+      <c r="O27" s="1"/>
+      <c r="P27" s="1"/>
+    </row>
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A28" s="1"/>
+      <c r="B28" s="1"/>
+      <c r="C28" s="1"/>
+      <c r="D28" s="1"/>
+      <c r="E28" s="1"/>
+      <c r="F28" s="1"/>
+      <c r="G28" s="1"/>
+      <c r="H28" s="1"/>
+      <c r="I28" s="1"/>
+      <c r="J28" s="1"/>
+      <c r="K28" s="1"/>
+      <c r="L28" s="1"/>
+      <c r="M28" s="1"/>
+      <c r="N28" s="1"/>
+      <c r="O28" s="1"/>
+      <c r="P28" s="1"/>
+    </row>
+    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A29" s="1"/>
+      <c r="B29" s="1"/>
+      <c r="C29" s="1"/>
+      <c r="D29" s="1"/>
+      <c r="E29" s="1"/>
+      <c r="F29" s="1"/>
+      <c r="G29" s="1"/>
+      <c r="H29" s="1"/>
+      <c r="I29" s="1"/>
+      <c r="J29" s="1"/>
+      <c r="K29" s="1"/>
+      <c r="L29" s="1"/>
+      <c r="M29" s="1"/>
+      <c r="N29" s="1"/>
+      <c r="O29" s="1"/>
+      <c r="P29" s="1"/>
+    </row>
+    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A30" s="1"/>
+      <c r="B30" s="1"/>
+      <c r="C30" s="1"/>
+      <c r="D30" s="1"/>
+      <c r="E30" s="1"/>
+      <c r="F30" s="1"/>
+      <c r="G30" s="1"/>
+      <c r="H30" s="1"/>
+      <c r="I30" s="1"/>
+      <c r="J30" s="1"/>
+      <c r="K30" s="1"/>
+      <c r="L30" s="1"/>
+      <c r="M30" s="1"/>
+      <c r="N30" s="1"/>
+      <c r="O30" s="1"/>
+      <c r="P30" s="1"/>
+    </row>
+    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A31" s="1"/>
+      <c r="B31" s="1"/>
+      <c r="C31" s="1"/>
+      <c r="D31" s="1"/>
+      <c r="E31" s="1"/>
+      <c r="F31" s="1"/>
+      <c r="G31" s="1"/>
+      <c r="H31" s="1"/>
+      <c r="I31" s="1"/>
+      <c r="J31" s="1"/>
+      <c r="K31" s="1"/>
+      <c r="L31" s="1"/>
+      <c r="M31" s="1"/>
+      <c r="N31" s="1"/>
+      <c r="O31" s="1"/>
+      <c r="P31" s="1"/>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="A2:XFD31">
     <cfRule type="cellIs" dxfId="35" priority="1" operator="equal">
       <formula>"No"</formula>
     </cfRule>
@@ -5836,25 +8313,12 @@
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q2:XFD2 A13:XFD33 P3:XFD12">
-    <cfRule type="cellIs" dxfId="32" priority="10" operator="equal">
-      <formula>"No"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="31" priority="11" operator="equal">
-      <formula>"Yes"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q2:XFD2 A13:XFD33 P3:XFD12">
-    <cfRule type="expression" dxfId="30" priority="12">
-      <formula>MOD(ROW(), 2) = 0</formula>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A665A9A6-A955-425D-A292-ED453B420318}">
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16921A6F-7CB8-4ECC-B4F3-AFD04063C385}">
   <dimension ref="A1:P33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -5926,7 +8390,7 @@
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>65</v>
+        <v>77</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>3</v>
@@ -5976,7 +8440,7 @@
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>3</v>
@@ -6009,7 +8473,7 @@
         <v>3</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="M3" s="1" t="s">
         <v>3</v>
@@ -6018,15 +8482,15 @@
         <v>3</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>0</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>3</v>
@@ -6068,114 +8532,60 @@
         <v>3</v>
       </c>
       <c r="O4" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="P4" s="1" t="s">
-        <v>0</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="L5" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="M5" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="N5" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="O5" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="P5" s="1" t="s">
-        <v>0</v>
-      </c>
+        <v>85</v>
+      </c>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
+      <c r="J5" s="1"/>
+      <c r="K5" s="1"/>
+      <c r="L5" s="1"/>
+      <c r="M5" s="1"/>
+      <c r="N5" s="1"/>
+      <c r="O5" s="1"/>
+      <c r="P5" s="1"/>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="L6" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="M6" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="N6" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="O6" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="P6" s="1" t="s">
-        <v>0</v>
-      </c>
+        <v>81</v>
+      </c>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
+      <c r="N6" s="1"/>
+      <c r="O6" s="1"/>
+      <c r="P6" s="1"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A7" s="1"/>
+      <c r="A7" s="1" t="s">
+        <v>82</v>
+      </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
@@ -6193,7 +8603,9 @@
       <c r="P7" s="1"/>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A8" s="1"/>
+      <c r="A8" s="1" t="s">
+        <v>83</v>
+      </c>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
@@ -6662,13 +9074,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:XFD33">
-    <cfRule type="cellIs" dxfId="29" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="1" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="27" priority="3">
+    <cfRule type="expression" dxfId="3" priority="3">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6676,7 +9088,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2BC1F7B8-E9E3-4996-94BF-2F4D98772BE4}">
   <dimension ref="A1:P33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -7358,13 +9770,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:XFD33">
-    <cfRule type="cellIs" dxfId="26" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="32" priority="1" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="31" priority="2" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="24" priority="3">
+    <cfRule type="expression" dxfId="30" priority="3">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7372,7 +9784,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50B60845-B986-4971-AC1C-D231CB8E9BF9}">
   <dimension ref="A1:P33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -8054,13 +10466,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:XFD33">
-    <cfRule type="cellIs" dxfId="23" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="29" priority="1" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="28" priority="2" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="21" priority="3">
+    <cfRule type="expression" dxfId="27" priority="3">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8068,8 +10480,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88E4E354-CC46-4D69-85EF-A6DDA23BD060}">
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC2183BA-4B28-4F00-8FAE-962779201001}">
   <dimension ref="A1:P33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -8087,7 +10499,6 @@
     <col min="12" max="12" width="10.28515625" customWidth="1"/>
     <col min="13" max="13" width="9.42578125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="11" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="8.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" s="3" customFormat="1" ht="60" x14ac:dyDescent="0.25">
@@ -8131,7 +10542,7 @@
         <v>16</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="O1" s="2" t="s">
         <v>64</v>
@@ -8142,7 +10553,7 @@
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>59</v>
+        <v>84</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>3</v>
@@ -8187,7 +10598,7 @@
         <v>3</v>
       </c>
       <c r="P2" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
@@ -8750,709 +11161,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:XFD33">
-    <cfRule type="cellIs" dxfId="20" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="19" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="18" priority="3">
-      <formula>MOD(ROW(), 2) = 0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2C91933-1FED-40CE-A7F7-694A14E79AF4}">
-  <dimension ref="A1:P33"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="27.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.28515625" customWidth="1"/>
-    <col min="4" max="4" width="9" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.28515625" customWidth="1"/>
-    <col min="13" max="13" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="8.140625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:16" s="3" customFormat="1" ht="60" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="O1" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="P1" s="2" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="N2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="O2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="P2" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-      <c r="K3" s="1"/>
-      <c r="L3" s="1"/>
-      <c r="M3" s="1"/>
-      <c r="N3" s="1"/>
-      <c r="O3" s="1"/>
-      <c r="P3" s="1"/>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-      <c r="J4" s="1"/>
-      <c r="K4" s="1"/>
-      <c r="L4" s="1"/>
-      <c r="M4" s="1"/>
-      <c r="N4" s="1"/>
-      <c r="O4" s="1"/>
-      <c r="P4" s="1"/>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
-      <c r="J5" s="1"/>
-      <c r="K5" s="1"/>
-      <c r="L5" s="1"/>
-      <c r="M5" s="1"/>
-      <c r="N5" s="1"/>
-      <c r="O5" s="1"/>
-      <c r="P5" s="1"/>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
-      <c r="J6" s="1"/>
-      <c r="K6" s="1"/>
-      <c r="L6" s="1"/>
-      <c r="M6" s="1"/>
-      <c r="N6" s="1"/>
-      <c r="O6" s="1"/>
-      <c r="P6" s="1"/>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
-      <c r="J7" s="1"/>
-      <c r="K7" s="1"/>
-      <c r="L7" s="1"/>
-      <c r="M7" s="1"/>
-      <c r="N7" s="1"/>
-      <c r="O7" s="1"/>
-      <c r="P7" s="1"/>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
-      <c r="G8" s="1"/>
-      <c r="H8" s="1"/>
-      <c r="I8" s="1"/>
-      <c r="J8" s="1"/>
-      <c r="K8" s="1"/>
-      <c r="L8" s="1"/>
-      <c r="M8" s="1"/>
-      <c r="N8" s="1"/>
-      <c r="O8" s="1"/>
-      <c r="P8" s="1"/>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
-      <c r="G9" s="1"/>
-      <c r="H9" s="1"/>
-      <c r="I9" s="1"/>
-      <c r="J9" s="1"/>
-      <c r="K9" s="1"/>
-      <c r="L9" s="1"/>
-      <c r="M9" s="1"/>
-      <c r="N9" s="1"/>
-      <c r="O9" s="1"/>
-      <c r="P9" s="1"/>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
-      <c r="G10" s="1"/>
-      <c r="H10" s="1"/>
-      <c r="I10" s="1"/>
-      <c r="J10" s="1"/>
-      <c r="K10" s="1"/>
-      <c r="L10" s="1"/>
-      <c r="M10" s="1"/>
-      <c r="N10" s="1"/>
-      <c r="O10" s="1"/>
-      <c r="P10" s="1"/>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
-      <c r="G11" s="1"/>
-      <c r="H11" s="1"/>
-      <c r="I11" s="1"/>
-      <c r="J11" s="1"/>
-      <c r="K11" s="1"/>
-      <c r="L11" s="1"/>
-      <c r="M11" s="1"/>
-      <c r="N11" s="1"/>
-      <c r="O11" s="1"/>
-      <c r="P11" s="1"/>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1"/>
-      <c r="G12" s="1"/>
-      <c r="H12" s="1"/>
-      <c r="I12" s="1"/>
-      <c r="J12" s="1"/>
-      <c r="K12" s="1"/>
-      <c r="L12" s="1"/>
-      <c r="M12" s="1"/>
-      <c r="N12" s="1"/>
-      <c r="O12" s="1"/>
-      <c r="P12" s="1"/>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="F13" s="1"/>
-      <c r="G13" s="1"/>
-      <c r="H13" s="1"/>
-      <c r="I13" s="1"/>
-      <c r="J13" s="1"/>
-      <c r="K13" s="1"/>
-      <c r="L13" s="1"/>
-      <c r="M13" s="1"/>
-      <c r="N13" s="1"/>
-      <c r="O13" s="1"/>
-      <c r="P13" s="1"/>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
-      <c r="G14" s="1"/>
-      <c r="H14" s="1"/>
-      <c r="I14" s="1"/>
-      <c r="J14" s="1"/>
-      <c r="K14" s="1"/>
-      <c r="L14" s="1"/>
-      <c r="M14" s="1"/>
-      <c r="N14" s="1"/>
-      <c r="O14" s="1"/>
-      <c r="P14" s="1"/>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
-      <c r="G15" s="1"/>
-      <c r="H15" s="1"/>
-      <c r="I15" s="1"/>
-      <c r="J15" s="1"/>
-      <c r="K15" s="1"/>
-      <c r="L15" s="1"/>
-      <c r="M15" s="1"/>
-      <c r="N15" s="1"/>
-      <c r="O15" s="1"/>
-      <c r="P15" s="1"/>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
-      <c r="G16" s="1"/>
-      <c r="H16" s="1"/>
-      <c r="I16" s="1"/>
-      <c r="J16" s="1"/>
-      <c r="K16" s="1"/>
-      <c r="L16" s="1"/>
-      <c r="M16" s="1"/>
-      <c r="N16" s="1"/>
-      <c r="O16" s="1"/>
-      <c r="P16" s="1"/>
-    </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
-      <c r="G17" s="1"/>
-      <c r="H17" s="1"/>
-      <c r="I17" s="1"/>
-      <c r="J17" s="1"/>
-      <c r="K17" s="1"/>
-      <c r="L17" s="1"/>
-      <c r="M17" s="1"/>
-      <c r="N17" s="1"/>
-      <c r="O17" s="1"/>
-      <c r="P17" s="1"/>
-    </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
-      <c r="F18" s="1"/>
-      <c r="G18" s="1"/>
-      <c r="H18" s="1"/>
-      <c r="I18" s="1"/>
-      <c r="J18" s="1"/>
-      <c r="K18" s="1"/>
-      <c r="L18" s="1"/>
-      <c r="M18" s="1"/>
-      <c r="N18" s="1"/>
-      <c r="O18" s="1"/>
-      <c r="P18" s="1"/>
-    </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A19" s="1"/>
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
-      <c r="F19" s="1"/>
-      <c r="G19" s="1"/>
-      <c r="H19" s="1"/>
-      <c r="I19" s="1"/>
-      <c r="J19" s="1"/>
-      <c r="K19" s="1"/>
-      <c r="L19" s="1"/>
-      <c r="M19" s="1"/>
-      <c r="N19" s="1"/>
-      <c r="O19" s="1"/>
-      <c r="P19" s="1"/>
-    </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
-      <c r="F20" s="1"/>
-      <c r="G20" s="1"/>
-      <c r="H20" s="1"/>
-      <c r="I20" s="1"/>
-      <c r="J20" s="1"/>
-      <c r="K20" s="1"/>
-      <c r="L20" s="1"/>
-      <c r="M20" s="1"/>
-      <c r="N20" s="1"/>
-      <c r="O20" s="1"/>
-      <c r="P20" s="1"/>
-    </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A21" s="1"/>
-      <c r="B21" s="1"/>
-      <c r="C21" s="1"/>
-      <c r="D21" s="1"/>
-      <c r="E21" s="1"/>
-      <c r="F21" s="1"/>
-      <c r="G21" s="1"/>
-      <c r="H21" s="1"/>
-      <c r="I21" s="1"/>
-      <c r="J21" s="1"/>
-      <c r="K21" s="1"/>
-      <c r="L21" s="1"/>
-      <c r="M21" s="1"/>
-      <c r="N21" s="1"/>
-      <c r="O21" s="1"/>
-      <c r="P21" s="1"/>
-    </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A22" s="1"/>
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
-      <c r="G22" s="1"/>
-      <c r="H22" s="1"/>
-      <c r="I22" s="1"/>
-      <c r="J22" s="1"/>
-      <c r="K22" s="1"/>
-      <c r="L22" s="1"/>
-      <c r="M22" s="1"/>
-      <c r="N22" s="1"/>
-      <c r="O22" s="1"/>
-      <c r="P22" s="1"/>
-    </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A23" s="1"/>
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
-      <c r="E23" s="1"/>
-      <c r="F23" s="1"/>
-      <c r="G23" s="1"/>
-      <c r="H23" s="1"/>
-      <c r="I23" s="1"/>
-      <c r="J23" s="1"/>
-      <c r="K23" s="1"/>
-      <c r="L23" s="1"/>
-      <c r="M23" s="1"/>
-      <c r="N23" s="1"/>
-      <c r="O23" s="1"/>
-      <c r="P23" s="1"/>
-    </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A24" s="1"/>
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
-      <c r="D24" s="1"/>
-      <c r="E24" s="1"/>
-      <c r="F24" s="1"/>
-      <c r="G24" s="1"/>
-      <c r="H24" s="1"/>
-      <c r="I24" s="1"/>
-      <c r="J24" s="1"/>
-      <c r="K24" s="1"/>
-      <c r="L24" s="1"/>
-      <c r="M24" s="1"/>
-      <c r="N24" s="1"/>
-      <c r="O24" s="1"/>
-      <c r="P24" s="1"/>
-    </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A25" s="1"/>
-      <c r="B25" s="1"/>
-      <c r="C25" s="1"/>
-      <c r="D25" s="1"/>
-      <c r="E25" s="1"/>
-      <c r="F25" s="1"/>
-      <c r="G25" s="1"/>
-      <c r="H25" s="1"/>
-      <c r="I25" s="1"/>
-      <c r="J25" s="1"/>
-      <c r="K25" s="1"/>
-      <c r="L25" s="1"/>
-      <c r="M25" s="1"/>
-      <c r="N25" s="1"/>
-      <c r="O25" s="1"/>
-      <c r="P25" s="1"/>
-    </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A26" s="1"/>
-      <c r="B26" s="1"/>
-      <c r="C26" s="1"/>
-      <c r="D26" s="1"/>
-      <c r="E26" s="1"/>
-      <c r="F26" s="1"/>
-      <c r="G26" s="1"/>
-      <c r="H26" s="1"/>
-      <c r="I26" s="1"/>
-      <c r="J26" s="1"/>
-      <c r="K26" s="1"/>
-      <c r="L26" s="1"/>
-      <c r="M26" s="1"/>
-      <c r="N26" s="1"/>
-      <c r="O26" s="1"/>
-      <c r="P26" s="1"/>
-    </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A27" s="1"/>
-      <c r="B27" s="1"/>
-      <c r="C27" s="1"/>
-      <c r="D27" s="1"/>
-      <c r="E27" s="1"/>
-      <c r="F27" s="1"/>
-      <c r="G27" s="1"/>
-      <c r="H27" s="1"/>
-      <c r="I27" s="1"/>
-      <c r="J27" s="1"/>
-      <c r="K27" s="1"/>
-      <c r="L27" s="1"/>
-      <c r="M27" s="1"/>
-      <c r="N27" s="1"/>
-      <c r="O27" s="1"/>
-      <c r="P27" s="1"/>
-    </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A28" s="1"/>
-      <c r="B28" s="1"/>
-      <c r="C28" s="1"/>
-      <c r="D28" s="1"/>
-      <c r="E28" s="1"/>
-      <c r="F28" s="1"/>
-      <c r="G28" s="1"/>
-      <c r="H28" s="1"/>
-      <c r="I28" s="1"/>
-      <c r="J28" s="1"/>
-      <c r="K28" s="1"/>
-      <c r="L28" s="1"/>
-      <c r="M28" s="1"/>
-      <c r="N28" s="1"/>
-      <c r="O28" s="1"/>
-      <c r="P28" s="1"/>
-    </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A29" s="1"/>
-      <c r="B29" s="1"/>
-      <c r="C29" s="1"/>
-      <c r="D29" s="1"/>
-      <c r="E29" s="1"/>
-      <c r="F29" s="1"/>
-      <c r="G29" s="1"/>
-      <c r="H29" s="1"/>
-      <c r="I29" s="1"/>
-      <c r="J29" s="1"/>
-      <c r="K29" s="1"/>
-      <c r="L29" s="1"/>
-      <c r="M29" s="1"/>
-      <c r="N29" s="1"/>
-      <c r="O29" s="1"/>
-      <c r="P29" s="1"/>
-    </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A30" s="1"/>
-      <c r="B30" s="1"/>
-      <c r="C30" s="1"/>
-      <c r="D30" s="1"/>
-      <c r="E30" s="1"/>
-      <c r="F30" s="1"/>
-      <c r="G30" s="1"/>
-      <c r="H30" s="1"/>
-      <c r="I30" s="1"/>
-      <c r="J30" s="1"/>
-      <c r="K30" s="1"/>
-      <c r="L30" s="1"/>
-      <c r="M30" s="1"/>
-      <c r="N30" s="1"/>
-      <c r="O30" s="1"/>
-      <c r="P30" s="1"/>
-    </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A31" s="1"/>
-      <c r="B31" s="1"/>
-      <c r="C31" s="1"/>
-      <c r="D31" s="1"/>
-      <c r="E31" s="1"/>
-      <c r="F31" s="1"/>
-      <c r="G31" s="1"/>
-      <c r="H31" s="1"/>
-      <c r="I31" s="1"/>
-      <c r="J31" s="1"/>
-      <c r="K31" s="1"/>
-      <c r="L31" s="1"/>
-      <c r="M31" s="1"/>
-      <c r="N31" s="1"/>
-      <c r="O31" s="1"/>
-      <c r="P31" s="1"/>
-    </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A32" s="1"/>
-      <c r="B32" s="1"/>
-      <c r="C32" s="1"/>
-      <c r="D32" s="1"/>
-      <c r="E32" s="1"/>
-      <c r="F32" s="1"/>
-      <c r="G32" s="1"/>
-      <c r="H32" s="1"/>
-      <c r="I32" s="1"/>
-      <c r="J32" s="1"/>
-      <c r="K32" s="1"/>
-      <c r="L32" s="1"/>
-      <c r="M32" s="1"/>
-      <c r="N32" s="1"/>
-      <c r="O32" s="1"/>
-      <c r="P32" s="1"/>
-    </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A33" s="1"/>
-      <c r="B33" s="1"/>
-      <c r="C33" s="1"/>
-      <c r="D33" s="1"/>
-      <c r="E33" s="1"/>
-      <c r="F33" s="1"/>
-      <c r="G33" s="1"/>
-      <c r="H33" s="1"/>
-      <c r="I33" s="1"/>
-      <c r="J33" s="1"/>
-      <c r="K33" s="1"/>
-      <c r="L33" s="1"/>
-      <c r="M33" s="1"/>
-      <c r="N33" s="1"/>
-      <c r="O33" s="1"/>
-      <c r="P33" s="1"/>
-    </row>
-  </sheetData>
-  <conditionalFormatting sqref="A2:XFD33">
-    <cfRule type="cellIs" dxfId="17" priority="1" operator="equal">
-      <formula>"No"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="2" operator="equal">
-      <formula>"Yes"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="15" priority="3">
+    <cfRule type="expression" dxfId="0" priority="3">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
fixed peak and rms leveling
</commit_message>
<xml_diff>
--- a/docs/excel_files/Ricks Music progress.xlsx
+++ b/docs/excel_files/Ricks Music progress.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MusicProcessing\docs\excel_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE84A0F8-F95E-4C0C-B393-AD57A92A32D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C07D467E-A059-4EFD-A76D-1D3932C95F26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="23016" yWindow="12768" windowWidth="23256" windowHeight="12576" activeTab="5" xr2:uid="{D1BCA01E-EFE2-441C-AE68-802A69D25AC4}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1190" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1249" uniqueCount="86">
   <si>
     <t>NA</t>
   </si>
@@ -303,7 +303,7 @@
     <t>Olivia Newton John</t>
   </si>
   <si>
-    <t>at a single man</t>
+    <t>Elton John &amp; Leon Russell</t>
   </si>
 </sst>
 </file>
@@ -2064,13 +2064,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:XFD33">
-    <cfRule type="cellIs" dxfId="26" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="20" priority="1" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="19" priority="2" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="24" priority="3">
+    <cfRule type="expression" dxfId="18" priority="3">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2760,13 +2760,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:XFD33">
-    <cfRule type="cellIs" dxfId="23" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="17" priority="1" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="2" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="21" priority="3">
+    <cfRule type="expression" dxfId="15" priority="3">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3505,46 +3505,46 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A3:O3">
-    <cfRule type="cellIs" dxfId="20" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="14" priority="1" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="19" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="2" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="18" priority="3">
+    <cfRule type="expression" dxfId="12" priority="3">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:P2">
-    <cfRule type="cellIs" dxfId="17" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="11" priority="4" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="5" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="15" priority="6">
+    <cfRule type="expression" dxfId="9" priority="6">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A4:XFD34">
-    <cfRule type="cellIs" dxfId="14" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="10" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="11" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="12" priority="12">
+    <cfRule type="expression" dxfId="6" priority="12">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P2:XFD3">
-    <cfRule type="cellIs" dxfId="11" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="7" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="8" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="9">
+    <cfRule type="expression" dxfId="3" priority="9">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4233,13 +4233,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:XFD33">
-    <cfRule type="cellIs" dxfId="8" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="3">
+    <cfRule type="expression" dxfId="0" priority="3">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8319,7 +8319,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16921A6F-7CB8-4ECC-B4F3-AFD04063C385}">
-  <dimension ref="A1:P33"/>
+  <dimension ref="A1:P34"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.28515625" bestFit="1" customWidth="1"/>
@@ -8473,7 +8473,7 @@
         <v>3</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="M3" s="1" t="s">
         <v>3</v>
@@ -8482,7 +8482,7 @@
         <v>3</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="P3" s="1" t="s">
         <v>13</v>
@@ -8532,7 +8532,7 @@
         <v>3</v>
       </c>
       <c r="O4" s="1" t="s">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="P4" s="1" t="s">
         <v>13</v>
@@ -8543,87 +8543,205 @@
         <v>80</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="M5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="N5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="O5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="P5" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
-      <c r="J5" s="1"/>
-      <c r="K5" s="1"/>
-      <c r="L5" s="1"/>
-      <c r="M5" s="1"/>
-      <c r="N5" s="1"/>
-      <c r="O5" s="1"/>
-      <c r="P5" s="1"/>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
-      <c r="J6" s="1"/>
-      <c r="K6" s="1"/>
-      <c r="L6" s="1"/>
-      <c r="M6" s="1"/>
-      <c r="N6" s="1"/>
-      <c r="O6" s="1"/>
-      <c r="P6" s="1"/>
+        <v>85</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="M6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="N6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="O6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="P6" s="1" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
-      <c r="J7" s="1"/>
-      <c r="K7" s="1"/>
-      <c r="L7" s="1"/>
-      <c r="M7" s="1"/>
-      <c r="N7" s="1"/>
-      <c r="O7" s="1"/>
-      <c r="P7" s="1"/>
+        <v>81</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="M7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="N7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="P7" s="1" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="L8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="M8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="N8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="P8" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
-      <c r="G8" s="1"/>
-      <c r="H8" s="1"/>
-      <c r="I8" s="1"/>
-      <c r="J8" s="1"/>
-      <c r="K8" s="1"/>
-      <c r="L8" s="1"/>
-      <c r="M8" s="1"/>
-      <c r="N8" s="1"/>
-      <c r="O8" s="1"/>
-      <c r="P8" s="1"/>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
@@ -9072,15 +9190,33 @@
       <c r="O33" s="1"/>
       <c r="P33" s="1"/>
     </row>
+    <row r="34" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A34" s="1"/>
+      <c r="B34" s="1"/>
+      <c r="C34" s="1"/>
+      <c r="D34" s="1"/>
+      <c r="E34" s="1"/>
+      <c r="F34" s="1"/>
+      <c r="G34" s="1"/>
+      <c r="H34" s="1"/>
+      <c r="I34" s="1"/>
+      <c r="J34" s="1"/>
+      <c r="K34" s="1"/>
+      <c r="L34" s="1"/>
+      <c r="M34" s="1"/>
+      <c r="N34" s="1"/>
+      <c r="O34" s="1"/>
+      <c r="P34" s="1"/>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:XFD33">
-    <cfRule type="cellIs" dxfId="5" priority="1" operator="equal">
+  <conditionalFormatting sqref="A2:XFD34">
+    <cfRule type="cellIs" dxfId="32" priority="1" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="31" priority="2" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="3">
+    <cfRule type="expression" dxfId="30" priority="3">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9770,13 +9906,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:XFD33">
-    <cfRule type="cellIs" dxfId="32" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="29" priority="1" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="31" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="28" priority="2" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="30" priority="3">
+    <cfRule type="expression" dxfId="27" priority="3">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10466,13 +10602,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:XFD33">
-    <cfRule type="cellIs" dxfId="29" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="26" priority="1" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="25" priority="2" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="27" priority="3">
+    <cfRule type="expression" dxfId="24" priority="3">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11161,13 +11297,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:XFD33">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="23" priority="1" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="22" priority="2" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="3">
+    <cfRule type="expression" dxfId="21" priority="3">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
consolidate normalize-*-filenames to one def and updated tests
</commit_message>
<xml_diff>
--- a/docs/excel_files/Ricks Music progress.xlsx
+++ b/docs/excel_files/Ricks Music progress.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MusicProcessing\docs\excel_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C07D467E-A059-4EFD-A76D-1D3932C95F26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6DC19FF-044D-4A4F-B65D-F6F7B30702FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="23016" yWindow="12768" windowWidth="23256" windowHeight="12576" activeTab="5" xr2:uid="{D1BCA01E-EFE2-441C-AE68-802A69D25AC4}"/>
+    <workbookView xWindow="23016" yWindow="12768" windowWidth="23256" windowHeight="12576" activeTab="4" xr2:uid="{D1BCA01E-EFE2-441C-AE68-802A69D25AC4}"/>
   </bookViews>
   <sheets>
     <sheet name="#" sheetId="4" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1249" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1265" uniqueCount="87">
   <si>
     <t>NA</t>
   </si>
@@ -139,9 +139,6 @@
   </si>
   <si>
     <t>Barenaked Ladies</t>
-  </si>
-  <si>
-    <t>Beach Boys</t>
   </si>
   <si>
     <t>Bee Gees</t>
@@ -305,6 +302,12 @@
   <si>
     <t>Elton John &amp; Leon Russell</t>
   </si>
+  <si>
+    <t>The Beach Boys</t>
+  </si>
+  <si>
+    <t>Derek And The Dominos</t>
+  </si>
 </sst>
 </file>
 
@@ -373,7 +376,31 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="63">
+  <dxfs count="66">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i/>
+      </font>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -1213,7 +1240,7 @@
         <v>5</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>6</v>
@@ -1234,7 +1261,7 @@
         <v>7</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>14</v>
@@ -1246,13 +1273,13 @@
         <v>16</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
@@ -1357,24 +1384,24 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:XFD3">
-    <cfRule type="cellIs" dxfId="62" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="65" priority="4" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="61" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="64" priority="5" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="60" priority="6">
+    <cfRule type="expression" dxfId="63" priority="6">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O2:O3">
-    <cfRule type="cellIs" dxfId="59" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="62" priority="1" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="58" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="61" priority="2" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="57" priority="3">
+    <cfRule type="expression" dxfId="60" priority="3">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1412,7 +1439,7 @@
         <v>5</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>6</v>
@@ -1433,7 +1460,7 @@
         <v>7</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>14</v>
@@ -1445,18 +1472,18 @@
         <v>16</v>
       </c>
       <c r="N1" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="O1" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="O1" s="2" t="s">
-        <v>64</v>
-      </c>
       <c r="P1" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>3</v>
@@ -2064,13 +2091,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:XFD33">
-    <cfRule type="cellIs" dxfId="20" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="23" priority="1" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="19" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="22" priority="2" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="18" priority="3">
+    <cfRule type="expression" dxfId="21" priority="3">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2108,7 +2135,7 @@
         <v>5</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>6</v>
@@ -2129,7 +2156,7 @@
         <v>7</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>14</v>
@@ -2141,18 +2168,18 @@
         <v>16</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>3</v>
@@ -2760,13 +2787,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:XFD33">
-    <cfRule type="cellIs" dxfId="17" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="20" priority="1" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="19" priority="2" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="15" priority="3">
+    <cfRule type="expression" dxfId="18" priority="3">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2776,7 +2803,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{773E741D-F1A5-41A0-B656-3E8F5BB0844F}">
-  <dimension ref="A1:P34"/>
+  <dimension ref="A1:P35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.28515625" bestFit="1" customWidth="1"/>
@@ -2803,7 +2830,7 @@
         <v>5</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>6</v>
@@ -2824,7 +2851,7 @@
         <v>7</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>14</v>
@@ -2836,18 +2863,18 @@
         <v>16</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>52</v>
+        <v>85</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>3</v>
@@ -2892,12 +2919,12 @@
         <v>3</v>
       </c>
       <c r="P2" s="1" t="s">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>68</v>
+        <v>51</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>3</v>
@@ -2946,22 +2973,54 @@
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-      <c r="J4" s="1"/>
-      <c r="K4" s="1"/>
-      <c r="L4" s="1"/>
-      <c r="M4" s="1"/>
-      <c r="N4" s="1"/>
-      <c r="O4" s="1"/>
-      <c r="P4" s="1"/>
+      <c r="A4" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="P4" s="1" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -3503,48 +3562,77 @@
       <c r="O34" s="1"/>
       <c r="P34" s="1"/>
     </row>
+    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A35" s="1"/>
+      <c r="B35" s="1"/>
+      <c r="C35" s="1"/>
+      <c r="D35" s="1"/>
+      <c r="E35" s="1"/>
+      <c r="F35" s="1"/>
+      <c r="G35" s="1"/>
+      <c r="H35" s="1"/>
+      <c r="I35" s="1"/>
+      <c r="J35" s="1"/>
+      <c r="K35" s="1"/>
+      <c r="L35" s="1"/>
+      <c r="M35" s="1"/>
+      <c r="N35" s="1"/>
+      <c r="O35" s="1"/>
+      <c r="P35" s="1"/>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="A3:O3">
-    <cfRule type="cellIs" dxfId="14" priority="1" operator="equal">
+  <conditionalFormatting sqref="A4:O4">
+    <cfRule type="cellIs" dxfId="17" priority="7" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="8" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="12" priority="3">
+    <cfRule type="expression" dxfId="15" priority="9">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:P2">
-    <cfRule type="cellIs" dxfId="11" priority="4" operator="equal">
+  <conditionalFormatting sqref="A3:P3">
+    <cfRule type="cellIs" dxfId="14" priority="10" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="11" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="6">
+    <cfRule type="expression" dxfId="12" priority="12">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A4:XFD34">
-    <cfRule type="cellIs" dxfId="8" priority="10" operator="equal">
+  <conditionalFormatting sqref="A2:XFD2">
+    <cfRule type="cellIs" dxfId="11" priority="1" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="2" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="12">
+    <cfRule type="expression" dxfId="9" priority="3">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P2:XFD3">
-    <cfRule type="cellIs" dxfId="5" priority="7" operator="equal">
+  <conditionalFormatting sqref="A5:XFD35">
+    <cfRule type="cellIs" dxfId="8" priority="16" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="17" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="9">
+    <cfRule type="expression" dxfId="6" priority="18">
+      <formula>MOD(ROW(), 2) = 0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P3:XFD4">
+    <cfRule type="cellIs" dxfId="5" priority="13" operator="equal">
+      <formula>"No"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="14" operator="equal">
+      <formula>"Yes"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="3" priority="15">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3581,7 +3669,7 @@
         <v>5</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>6</v>
@@ -3602,7 +3690,7 @@
         <v>7</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>14</v>
@@ -3614,18 +3702,18 @@
         <v>16</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>13</v>
@@ -4274,7 +4362,7 @@
         <v>5</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>6</v>
@@ -4295,7 +4383,7 @@
         <v>7</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>14</v>
@@ -4307,13 +4395,13 @@
         <v>16</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
@@ -4768,7 +4856,7 @@
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>3</v>
@@ -4818,33 +4906,33 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:XFD11">
-    <cfRule type="cellIs" dxfId="56" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="59" priority="7" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="55" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="58" priority="8" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="54" priority="9">
+    <cfRule type="expression" dxfId="57" priority="9">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O2:O11">
-    <cfRule type="cellIs" dxfId="53" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="56" priority="1" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="52" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="55" priority="2" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="51" priority="3">
+    <cfRule type="expression" dxfId="54" priority="3">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="50" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="53" priority="4" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="49" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="52" priority="5" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="48" priority="6">
+    <cfRule type="expression" dxfId="51" priority="6">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4854,7 +4942,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67B08846-0C86-4F4B-BBEE-7D9E018F9FC5}">
-  <dimension ref="A1:P48"/>
+  <dimension ref="A1:P47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.28515625" bestFit="1" customWidth="1"/>
@@ -4882,7 +4970,7 @@
         <v>5</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>6</v>
@@ -4903,7 +4991,7 @@
         <v>7</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>14</v>
@@ -4915,13 +5003,13 @@
         <v>16</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
@@ -5126,7 +5214,7 @@
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>3</v>
@@ -5171,7 +5259,7 @@
         <v>3</v>
       </c>
       <c r="P6" s="1" t="s">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
@@ -5221,7 +5309,7 @@
         <v>3</v>
       </c>
       <c r="P7" s="1" t="s">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
@@ -5371,12 +5459,12 @@
         <v>3</v>
       </c>
       <c r="P10" s="1" t="s">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>3</v>
@@ -5421,7 +5509,7 @@
         <v>3</v>
       </c>
       <c r="P11" s="1" t="s">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
@@ -5476,7 +5564,7 @@
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>3</v>
@@ -5521,7 +5609,7 @@
         <v>3</v>
       </c>
       <c r="P13" s="1" t="s">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
@@ -5621,7 +5709,7 @@
         <v>3</v>
       </c>
       <c r="P15" s="1" t="s">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.25">
@@ -5675,54 +5763,22 @@
       </c>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="H17" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="I17" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="J17" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="K17" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="L17" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="M17" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="N17" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="O17" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="P17" s="1" t="s">
-        <v>3</v>
-      </c>
+      <c r="A17" s="1"/>
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
+      <c r="H17" s="1"/>
+      <c r="I17" s="1"/>
+      <c r="J17" s="1"/>
+      <c r="K17" s="1"/>
+      <c r="L17" s="1"/>
+      <c r="M17" s="1"/>
+      <c r="N17" s="1"/>
+      <c r="O17" s="1"/>
+      <c r="P17" s="1"/>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
@@ -6264,44 +6320,26 @@
       <c r="O47" s="1"/>
       <c r="P47" s="1"/>
     </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A48" s="1"/>
-      <c r="B48" s="1"/>
-      <c r="C48" s="1"/>
-      <c r="D48" s="1"/>
-      <c r="E48" s="1"/>
-      <c r="F48" s="1"/>
-      <c r="G48" s="1"/>
-      <c r="H48" s="1"/>
-      <c r="I48" s="1"/>
-      <c r="J48" s="1"/>
-      <c r="K48" s="1"/>
-      <c r="L48" s="1"/>
-      <c r="M48" s="1"/>
-      <c r="N48" s="1"/>
-      <c r="O48" s="1"/>
-      <c r="P48" s="1"/>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:O48 Q2:XFD48 N18:P48">
-    <cfRule type="cellIs" dxfId="47" priority="4" operator="equal">
+  <conditionalFormatting sqref="A2:O47 Q2:XFD47 N17:P47">
+    <cfRule type="cellIs" dxfId="50" priority="4" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="46" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="49" priority="5" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="45" priority="6">
+    <cfRule type="expression" dxfId="48" priority="6">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P2:P17">
-    <cfRule type="cellIs" dxfId="44" priority="1" operator="equal">
+  <conditionalFormatting sqref="P2:P16">
+    <cfRule type="cellIs" dxfId="47" priority="1" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="43" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="46" priority="2" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="42" priority="3">
+    <cfRule type="expression" dxfId="45" priority="3">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6339,7 +6377,7 @@
         <v>5</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>6</v>
@@ -6360,7 +6398,7 @@
         <v>7</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>14</v>
@@ -6372,18 +6410,18 @@
         <v>16</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>3</v>
@@ -6433,7 +6471,7 @@
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>3</v>
@@ -6483,7 +6521,7 @@
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>3</v>
@@ -6533,7 +6571,7 @@
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>3</v>
@@ -6583,7 +6621,7 @@
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>3</v>
@@ -6633,7 +6671,7 @@
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>3</v>
@@ -6683,7 +6721,7 @@
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>3</v>
@@ -6733,7 +6771,7 @@
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>3</v>
@@ -6833,7 +6871,7 @@
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>3</v>
@@ -6883,7 +6921,7 @@
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>3</v>
@@ -7311,26 +7349,26 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:P12">
-    <cfRule type="cellIs" dxfId="41" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="44" priority="1" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="40" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="43" priority="2" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="39" priority="3">
+    <cfRule type="expression" dxfId="42" priority="3">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P3:XFD12 Q2:XFD2 A13:XFD33">
-    <cfRule type="cellIs" dxfId="38" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="41" priority="10" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="37" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="40" priority="11" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q2:XFD2 P3:XFD12 A13:XFD33">
-    <cfRule type="expression" dxfId="36" priority="12">
+    <cfRule type="expression" dxfId="39" priority="12">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7340,7 +7378,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A665A9A6-A955-425D-A292-ED453B420318}">
-  <dimension ref="A1:P31"/>
+  <dimension ref="A1:P32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.28515625" bestFit="1" customWidth="1"/>
@@ -7367,7 +7405,7 @@
         <v>5</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>6</v>
@@ -7388,7 +7426,7 @@
         <v>7</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>14</v>
@@ -7400,18 +7438,18 @@
         <v>16</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>3</v>
@@ -7461,7 +7499,7 @@
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>3</v>
@@ -7511,7 +7549,7 @@
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>3</v>
@@ -7561,7 +7599,7 @@
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>3</v>
@@ -7611,7 +7649,7 @@
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>3</v>
@@ -7661,7 +7699,7 @@
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>71</v>
+        <v>86</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>3</v>
@@ -7706,12 +7744,12 @@
         <v>3</v>
       </c>
       <c r="P7" s="1" t="s">
-        <v>13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>3</v>
@@ -7761,7 +7799,7 @@
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>3</v>
@@ -7811,7 +7849,7 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>3</v>
@@ -7856,12 +7894,12 @@
         <v>3</v>
       </c>
       <c r="P10" s="1" t="s">
-        <v>0</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>3</v>
@@ -7911,7 +7949,7 @@
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>3</v>
@@ -7956,26 +7994,58 @@
         <v>3</v>
       </c>
       <c r="P12" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="K13" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="L13" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="M13" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="N13" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="O13" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="P13" s="1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="F13" s="1"/>
-      <c r="G13" s="1"/>
-      <c r="H13" s="1"/>
-      <c r="I13" s="1"/>
-      <c r="J13" s="1"/>
-      <c r="K13" s="1"/>
-      <c r="L13" s="1"/>
-      <c r="M13" s="1"/>
-      <c r="N13" s="1"/>
-      <c r="O13" s="1"/>
-      <c r="P13" s="1"/>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
@@ -8301,15 +8371,33 @@
       <c r="O31" s="1"/>
       <c r="P31" s="1"/>
     </row>
+    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A32" s="1"/>
+      <c r="B32" s="1"/>
+      <c r="C32" s="1"/>
+      <c r="D32" s="1"/>
+      <c r="E32" s="1"/>
+      <c r="F32" s="1"/>
+      <c r="G32" s="1"/>
+      <c r="H32" s="1"/>
+      <c r="I32" s="1"/>
+      <c r="J32" s="1"/>
+      <c r="K32" s="1"/>
+      <c r="L32" s="1"/>
+      <c r="M32" s="1"/>
+      <c r="N32" s="1"/>
+      <c r="O32" s="1"/>
+      <c r="P32" s="1"/>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:XFD31">
-    <cfRule type="cellIs" dxfId="35" priority="1" operator="equal">
+  <conditionalFormatting sqref="A2:XFD32">
+    <cfRule type="cellIs" dxfId="38" priority="1" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="34" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="37" priority="2" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="33" priority="3">
+    <cfRule type="expression" dxfId="36" priority="3">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8346,7 +8434,7 @@
         <v>5</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>6</v>
@@ -8367,7 +8455,7 @@
         <v>7</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>14</v>
@@ -8379,18 +8467,18 @@
         <v>16</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>3</v>
@@ -8440,7 +8528,7 @@
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>3</v>
@@ -8490,7 +8578,7 @@
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>3</v>
@@ -8540,7 +8628,7 @@
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>3</v>
@@ -8590,7 +8678,7 @@
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>3</v>
@@ -8640,7 +8728,7 @@
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>3</v>
@@ -8690,7 +8778,7 @@
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>3</v>
@@ -8740,7 +8828,7 @@
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -9210,13 +9298,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:XFD34">
-    <cfRule type="cellIs" dxfId="32" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="35" priority="1" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="31" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="34" priority="2" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="30" priority="3">
+    <cfRule type="expression" dxfId="33" priority="3">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9254,7 +9342,7 @@
         <v>5</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>6</v>
@@ -9275,7 +9363,7 @@
         <v>7</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>14</v>
@@ -9287,13 +9375,13 @@
         <v>16</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
@@ -9906,13 +9994,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:XFD33">
-    <cfRule type="cellIs" dxfId="29" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="32" priority="1" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="31" priority="2" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="27" priority="3">
+    <cfRule type="expression" dxfId="30" priority="3">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9950,7 +10038,7 @@
         <v>5</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>6</v>
@@ -9971,7 +10059,7 @@
         <v>7</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>14</v>
@@ -9983,13 +10071,13 @@
         <v>16</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
@@ -10602,13 +10690,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:XFD33">
-    <cfRule type="cellIs" dxfId="26" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="29" priority="1" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="28" priority="2" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="24" priority="3">
+    <cfRule type="expression" dxfId="27" priority="3">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10645,7 +10733,7 @@
         <v>5</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>6</v>
@@ -10666,7 +10754,7 @@
         <v>7</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>14</v>
@@ -10678,18 +10766,18 @@
         <v>16</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>3</v>
@@ -11297,13 +11385,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:XFD33">
-    <cfRule type="cellIs" dxfId="23" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="26" priority="1" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="25" priority="2" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="21" priority="3">
+    <cfRule type="expression" dxfId="24" priority="3">
       <formula>MOD(ROW(), 2) = 0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
clean up and re-org
</commit_message>
<xml_diff>
--- a/docs/excel_files/Ricks Music progress.xlsx
+++ b/docs/excel_files/Ricks Music progress.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MusicProcessing\docs\excel_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DA664B9-4590-424D-B822-C921EBDF1DD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A934227C-7D8C-4299-9221-B33DDD928869}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="23016" yWindow="12768" windowWidth="23256" windowHeight="12576" activeTab="5" xr2:uid="{D1BCA01E-EFE2-441C-AE68-802A69D25AC4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="5" xr2:uid="{D1BCA01E-EFE2-441C-AE68-802A69D25AC4}"/>
   </bookViews>
   <sheets>
     <sheet name="#" sheetId="4" r:id="rId1"/>
@@ -315,7 +315,7 @@
     <t>Arthur Lewis</t>
   </si>
   <si>
-    <t>No reason To Cry</t>
+    <t>Old Sock</t>
   </si>
 </sst>
 </file>

</xml_diff>